<commit_message>
chore(data-release): publish site data 2026-08-20 02:00:34 UTC
</commit_message>
<xml_diff>
--- a/diseases/d001/2026-2029.xlsx
+++ b/diseases/d001/2026-2029.xlsx
@@ -10873,12 +10873,12 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>CN</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>China</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -10915,6 +10915,9 @@
         <v>0</v>
       </c>
       <c r="O71" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q71" t="n">
         <v>0</v>
       </c>
       <c r="R71" t="n">
@@ -10951,42 +10954,42 @@
       </c>
       <c r="AV71" t="inlineStr">
         <is>
-          <t>kdca_open_api</t>
+          <t>cdc_weekly</t>
         </is>
       </c>
       <c r="AW71" t="inlineStr">
         <is>
-          <t>Korea KDCA EID</t>
+          <t>China CDC Weekly</t>
         </is>
       </c>
       <c r="AX71" t="inlineStr">
         <is>
-          <t>https://www.data.go.kr/data/15139178/openapi.do</t>
+          <t>https://weekly.chinacdc.cn</t>
         </is>
       </c>
       <c r="AY71" t="inlineStr">
         <is>
-          <t>open_api_or_portal_download</t>
+          <t>web</t>
         </is>
       </c>
       <c r="AZ71" t="inlineStr">
         <is>
-          <t>kdca_open_api</t>
+          <t>cdc_weekly; nhc; pubmed</t>
         </is>
       </c>
       <c r="BA71" t="inlineStr">
         <is>
-          <t>Korea KDCA EID</t>
+          <t>China CDC Weekly; National Disease Control and Prevention Administration; PubMed</t>
         </is>
       </c>
       <c r="BB71" t="inlineStr">
         <is>
-          <t>https://www.data.go.kr/data/15139178/openapi.do</t>
+          <t>https://weekly.chinacdc.cn; https://www.ndcpa.gov.cn; https://pubmed.ncbi.nlm.nih.gov</t>
         </is>
       </c>
       <c r="BC71" t="inlineStr">
         <is>
-          <t>open_api_or_portal_download</t>
+          <t>web; web; web</t>
         </is>
       </c>
     </row>
@@ -11018,12 +11021,12 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -11048,7 +11051,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="M72" t="inlineStr">
@@ -11096,42 +11099,42 @@
       </c>
       <c r="AV72" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>kdca_open_api</t>
         </is>
       </c>
       <c r="AW72" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>Korea KDCA EID</t>
         </is>
       </c>
       <c r="AX72" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://www.data.go.kr/data/15139178/openapi.do</t>
         </is>
       </c>
       <c r="AY72" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>open_api_or_portal_download</t>
         </is>
       </c>
       <c r="AZ72" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>kdca_open_api</t>
         </is>
       </c>
       <c r="BA72" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>Korea KDCA EID</t>
         </is>
       </c>
       <c r="BB72" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://www.data.go.kr/data/15139178/openapi.do</t>
         </is>
       </c>
       <c r="BC72" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>open_api_or_portal_download</t>
         </is>
       </c>
     </row>
@@ -11163,12 +11166,12 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -11241,42 +11244,42 @@
       </c>
       <c r="AV73" t="inlineStr">
         <is>
-          <t>nndss_api</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="AW73" t="inlineStr">
         <is>
-          <t>US CDC NNDSS</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="AX73" t="inlineStr">
         <is>
-          <t>https://data.cdc.gov/browse?category=NNDSS</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="AY73" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>web</t>
         </is>
       </c>
       <c r="AZ73" t="inlineStr">
         <is>
-          <t>nndss_api; nhss_hiv</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="BA73" t="inlineStr">
         <is>
-          <t>US CDC NNDSS; US CDC NHSS HIV</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="BB73" t="inlineStr">
         <is>
-          <t>https://data.cdc.gov/browse?category=NNDSS; https://www.cdc.gov/hiv-data/nhss/</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="BC73" t="inlineStr">
         <is>
-          <t>api; api</t>
+          <t>web</t>
         </is>
       </c>
     </row>
@@ -11308,12 +11311,12 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -11338,7 +11341,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="M74" t="inlineStr">
@@ -11386,42 +11389,42 @@
       </c>
       <c r="AV74" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>nndss_api</t>
         </is>
       </c>
       <c r="AW74" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>US CDC NNDSS</t>
         </is>
       </c>
       <c r="AX74" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://data.cdc.gov/browse?category=NNDSS</t>
         </is>
       </c>
       <c r="AY74" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>api</t>
         </is>
       </c>
       <c r="AZ74" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>nndss_api; nhss_hiv</t>
         </is>
       </c>
       <c r="BA74" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>US CDC NNDSS; US CDC NHSS HIV</t>
         </is>
       </c>
       <c r="BB74" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://data.cdc.gov/browse?category=NNDSS; https://www.cdc.gov/hiv-data/nhss/</t>
         </is>
       </c>
       <c r="BC74" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>api; api</t>
         </is>
       </c>
     </row>
@@ -11453,12 +11456,12 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -11531,42 +11534,42 @@
       </c>
       <c r="AV75" t="inlineStr">
         <is>
-          <t>nndss_api</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="AW75" t="inlineStr">
         <is>
-          <t>US CDC NNDSS</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="AX75" t="inlineStr">
         <is>
-          <t>https://data.cdc.gov/browse?category=NNDSS</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="AY75" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>web</t>
         </is>
       </c>
       <c r="AZ75" t="inlineStr">
         <is>
-          <t>nndss_api; nhss_hiv</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="BA75" t="inlineStr">
         <is>
-          <t>US CDC NNDSS; US CDC NHSS HIV</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="BB75" t="inlineStr">
         <is>
-          <t>https://data.cdc.gov/browse?category=NNDSS; https://www.cdc.gov/hiv-data/nhss/</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="BC75" t="inlineStr">
         <is>
-          <t>api; api</t>
+          <t>web</t>
         </is>
       </c>
     </row>
@@ -11598,12 +11601,12 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -11628,7 +11631,7 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="M76" t="inlineStr">
@@ -11676,42 +11679,42 @@
       </c>
       <c r="AV76" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>nndss_api</t>
         </is>
       </c>
       <c r="AW76" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>US CDC NNDSS</t>
         </is>
       </c>
       <c r="AX76" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://data.cdc.gov/browse?category=NNDSS</t>
         </is>
       </c>
       <c r="AY76" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>api</t>
         </is>
       </c>
       <c r="AZ76" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>nndss_api; nhss_hiv</t>
         </is>
       </c>
       <c r="BA76" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>US CDC NNDSS; US CDC NHSS HIV</t>
         </is>
       </c>
       <c r="BB76" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://data.cdc.gov/browse?category=NNDSS; https://www.cdc.gov/hiv-data/nhss/</t>
         </is>
       </c>
       <c r="BC76" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>api; api</t>
         </is>
       </c>
     </row>
@@ -11743,12 +11746,12 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -11821,42 +11824,42 @@
       </c>
       <c r="AV77" t="inlineStr">
         <is>
-          <t>nndss_api</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="AW77" t="inlineStr">
         <is>
-          <t>US CDC NNDSS</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="AX77" t="inlineStr">
         <is>
-          <t>https://data.cdc.gov/browse?category=NNDSS</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="AY77" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>web</t>
         </is>
       </c>
       <c r="AZ77" t="inlineStr">
         <is>
-          <t>nndss_api; nhss_hiv</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="BA77" t="inlineStr">
         <is>
-          <t>US CDC NNDSS; US CDC NHSS HIV</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="BB77" t="inlineStr">
         <is>
-          <t>https://data.cdc.gov/browse?category=NNDSS; https://www.cdc.gov/hiv-data/nhss/</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="BC77" t="inlineStr">
         <is>
-          <t>api; api</t>
+          <t>web</t>
         </is>
       </c>
     </row>
@@ -11888,12 +11891,12 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -11918,7 +11921,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -11966,42 +11969,42 @@
       </c>
       <c r="AV78" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>nndss_api</t>
         </is>
       </c>
       <c r="AW78" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>US CDC NNDSS</t>
         </is>
       </c>
       <c r="AX78" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://data.cdc.gov/browse?category=NNDSS</t>
         </is>
       </c>
       <c r="AY78" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>api</t>
         </is>
       </c>
       <c r="AZ78" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>nndss_api; nhss_hiv</t>
         </is>
       </c>
       <c r="BA78" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>US CDC NNDSS; US CDC NHSS HIV</t>
         </is>
       </c>
       <c r="BB78" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://data.cdc.gov/browse?category=NNDSS; https://www.cdc.gov/hiv-data/nhss/</t>
         </is>
       </c>
       <c r="BC78" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>api; api</t>
         </is>
       </c>
     </row>
@@ -12033,12 +12036,12 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -12111,42 +12114,42 @@
       </c>
       <c r="AV79" t="inlineStr">
         <is>
-          <t>nndss_api</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="AW79" t="inlineStr">
         <is>
-          <t>US CDC NNDSS</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="AX79" t="inlineStr">
         <is>
-          <t>https://data.cdc.gov/browse?category=NNDSS</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="AY79" t="inlineStr">
         <is>
-          <t>api</t>
+          <t>web</t>
         </is>
       </c>
       <c r="AZ79" t="inlineStr">
         <is>
-          <t>nndss_api; nhss_hiv</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="BA79" t="inlineStr">
         <is>
-          <t>US CDC NNDSS; US CDC NHSS HIV</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="BB79" t="inlineStr">
         <is>
-          <t>https://data.cdc.gov/browse?category=NNDSS; https://www.cdc.gov/hiv-data/nhss/</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="BC79" t="inlineStr">
         <is>
-          <t>api; api</t>
+          <t>web</t>
         </is>
       </c>
     </row>
@@ -12178,12 +12181,12 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>US</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">
@@ -12208,7 +12211,7 @@
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="M80" t="inlineStr">
@@ -12256,42 +12259,42 @@
       </c>
       <c r="AV80" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>nndss_api</t>
         </is>
       </c>
       <c r="AW80" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>US CDC NNDSS</t>
         </is>
       </c>
       <c r="AX80" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://data.cdc.gov/browse?category=NNDSS</t>
         </is>
       </c>
       <c r="AY80" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>api</t>
         </is>
       </c>
       <c r="AZ80" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>nndss_api; nhss_hiv</t>
         </is>
       </c>
       <c r="BA80" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>US CDC NNDSS; US CDC NHSS HIV</t>
         </is>
       </c>
       <c r="BB80" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://data.cdc.gov/browse?category=NNDSS; https://www.cdc.gov/hiv-data/nhss/</t>
         </is>
       </c>
       <c r="BC80" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>api; api</t>
         </is>
       </c>
     </row>
@@ -12323,12 +12326,12 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>KR</t>
+          <t>JP</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="H81" t="inlineStr">
@@ -12353,12 +12356,12 @@
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="M81" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>2026-07</t>
         </is>
       </c>
       <c r="N81" t="n">
@@ -12401,42 +12404,42 @@
       </c>
       <c r="AV81" t="inlineStr">
         <is>
-          <t>kdca_open_api</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="AW81" t="inlineStr">
         <is>
-          <t>Korea KDCA EID</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="AX81" t="inlineStr">
         <is>
-          <t>https://www.data.go.kr/data/15139178/openapi.do</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="AY81" t="inlineStr">
         <is>
-          <t>open_api_or_portal_download</t>
+          <t>web</t>
         </is>
       </c>
       <c r="AZ81" t="inlineStr">
         <is>
-          <t>kdca_open_api</t>
+          <t>jp_weekly</t>
         </is>
       </c>
       <c r="BA81" t="inlineStr">
         <is>
-          <t>Korea KDCA EID</t>
+          <t>JP NIID Weekly</t>
         </is>
       </c>
       <c r="BB81" t="inlineStr">
         <is>
-          <t>https://www.data.go.kr/data/15139178/openapi.do</t>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
         </is>
       </c>
       <c r="BC81" t="inlineStr">
         <is>
-          <t>open_api_or_portal_download</t>
+          <t>web</t>
         </is>
       </c>
     </row>
@@ -12468,12 +12471,12 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>JP</t>
+          <t>KR</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="H82" t="inlineStr">
@@ -12498,7 +12501,7 @@
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="M82" t="inlineStr">
@@ -12546,42 +12549,42 @@
       </c>
       <c r="AV82" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>kdca_open_api</t>
         </is>
       </c>
       <c r="AW82" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>Korea KDCA EID</t>
         </is>
       </c>
       <c r="AX82" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://www.data.go.kr/data/15139178/openapi.do</t>
         </is>
       </c>
       <c r="AY82" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>open_api_or_portal_download</t>
         </is>
       </c>
       <c r="AZ82" t="inlineStr">
         <is>
-          <t>jp_weekly</t>
+          <t>kdca_open_api</t>
         </is>
       </c>
       <c r="BA82" t="inlineStr">
         <is>
-          <t>JP NIID Weekly</t>
+          <t>Korea KDCA EID</t>
         </is>
       </c>
       <c r="BB82" t="inlineStr">
         <is>
-          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+          <t>https://www.data.go.kr/data/15139178/openapi.do</t>
         </is>
       </c>
       <c r="BC82" t="inlineStr">
         <is>
-          <t>web</t>
+          <t>open_api_or_portal_download</t>
         </is>
       </c>
     </row>
@@ -12643,7 +12646,7 @@
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-02</t>
         </is>
       </c>
       <c r="M83" t="inlineStr">
@@ -12725,6 +12728,151 @@
         </is>
       </c>
       <c r="BC83" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>disease</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>D001</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>plague</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Plague</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>JP</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>D001</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>Plague</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>鼠疫</t>
+        </is>
+      </c>
+      <c r="K84" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="N84" t="n">
+        <v>0</v>
+      </c>
+      <c r="O84" t="n">
+        <v>0</v>
+      </c>
+      <c r="R84" t="n">
+        <v>0</v>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="AO84" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AP84" t="inlineStr">
+        <is>
+          <t>legacy_fallback</t>
+        </is>
+      </c>
+      <c r="AR84" t="inlineStr">
+        <is>
+          <t>legacy_identity_may_be_lossy</t>
+        </is>
+      </c>
+      <c r="AS84" t="inlineStr"/>
+      <c r="AT84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU84" t="inlineStr">
+        <is>
+          <t>No eligible registered case-count series facts are available for this disease and country; the public curve uses the legacy flat table.</t>
+        </is>
+      </c>
+      <c r="AV84" t="inlineStr">
+        <is>
+          <t>jp_weekly</t>
+        </is>
+      </c>
+      <c r="AW84" t="inlineStr">
+        <is>
+          <t>JP NIID Weekly</t>
+        </is>
+      </c>
+      <c r="AX84" t="inlineStr">
+        <is>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+        </is>
+      </c>
+      <c r="AY84" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="AZ84" t="inlineStr">
+        <is>
+          <t>jp_weekly</t>
+        </is>
+      </c>
+      <c r="BA84" t="inlineStr">
+        <is>
+          <t>JP NIID Weekly</t>
+        </is>
+      </c>
+      <c r="BB84" t="inlineStr">
+        <is>
+          <t>https://id-info.jihs.go.jp/en/surveillance/idwr/rapid/index.html</t>
+        </is>
+      </c>
+      <c r="BC84" t="inlineStr">
         <is>
           <t>web</t>
         </is>
@@ -12846,7 +12994,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="10">
@@ -12856,7 +13004,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="11">

</xml_diff>